<commit_message>
Expand blind holdout to 11 verified samples
</commit_message>
<xml_diff>
--- a/outputs/holdout_v0_1/vibebench_blind_holdout_100_v0_1.xlsx
+++ b/outputs/holdout_v0_1/vibebench_blind_holdout_100_v0_1.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R5fecbe1f2d394be1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samples" sheetId="2" r:id="R05b3e337f7714b36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="3" r:id="R3774918122794eee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rf3a506fdcc944a67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra0919e19288a46d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samples" sheetId="2" r:id="R08c9a0a4b6454f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="3" r:id="Rc233e544ae18470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R89fa380ad9cc4624"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -447,7 +447,7 @@
       </x:c>
       <x:c r="B6" s="13" t="n">
         <x:f>COUNTIF('Samples'!M2:M101,"REACHABLE")+COUNTIF('Samples'!M2:M101,"FAILED")+COUNTIF('Samples'!M2:M101,"RETRY")</x:f>
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -456,7 +456,7 @@
       </x:c>
       <x:c r="B7" s="13" t="n">
         <x:f>COUNTIF('Samples'!S2:S101,"PASS")+COUNTIF('Samples'!S2:S101,"FAIL")</x:f>
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -465,7 +465,7 @@
       </x:c>
       <x:c r="B8" s="13" t="n">
         <x:f>COUNTIF('Samples'!M2:M101,"REACHABLE")</x:f>
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -474,7 +474,7 @@
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:f>COUNTIF('Samples'!T2:T101,"READY")</x:f>
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -483,7 +483,7 @@
       </x:c>
       <x:c r="B10" s="13" t="n">
         <x:f>COUNTIFS('Samples'!B2:B101,"AI",'Samples'!T2:T101,"READY")</x:f>
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -492,7 +492,7 @@
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:f>COUNTIFS('Samples'!B2:B101,"HUMAN",'Samples'!T2:T101,"READY")</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -529,11 +529,11 @@
       </x:c>
       <x:c r="C16" t="n">
         <x:f>COUNTIFS('Samples'!C2:C101,A16,'Samples'!M2:M101,"REACHABLE")+COUNTIFS('Samples'!C2:C101,A16,'Samples'!M2:M101,"FAILED")+COUNTIFS('Samples'!C2:C101,A16,'Samples'!M2:M101,"RETRY")</x:f>
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D16" t="n">
         <x:f>COUNTIFS('Samples'!C2:C101,A16,'Samples'!T2:T101,"READY")</x:f>
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -609,11 +609,11 @@
       </x:c>
       <x:c r="C21" t="n">
         <x:f>COUNTIFS('Samples'!C2:C101,A21,'Samples'!M2:M101,"REACHABLE")+COUNTIFS('Samples'!C2:C101,A21,'Samples'!M2:M101,"FAILED")+COUNTIFS('Samples'!C2:C101,A21,'Samples'!M2:M101,"RETRY")</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D21" t="n">
         <x:f>COUNTIFS('Samples'!C2:C101,A21,'Samples'!T2:T101,"READY")</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -900,34 +900,58 @@
       <x:c r="D3" s="17" t="str">
         <x:v>Lovable</x:v>
       </x:c>
-      <x:c r="E3" s="19" t="str"/>
-      <x:c r="F3" s="19" t="str"/>
-      <x:c r="G3" s="19" t="str"/>
-      <x:c r="H3" s="19" t="str"/>
-      <x:c r="I3" s="19" t="str"/>
-      <x:c r="J3" s="20" t="str"/>
-      <x:c r="K3" s="20" t="str"/>
-      <x:c r="L3" s="20" t="str"/>
+      <x:c r="E3" s="19" t="str">
+        <x:v>Community safety map</x:v>
+      </x:c>
+      <x:c r="F3" s="19" t="str">
+        <x:v>https://safety-sentinel-guard.lovable.app/</x:v>
+      </x:c>
+      <x:c r="G3" s="19" t="str">
+        <x:v>https://lovable.dev/blog/2025-01-17-mysafe-x-lovable-hackathon-canada-winner</x:v>
+      </x:c>
+      <x:c r="H3" s="19" t="str">
+        <x:v>official_builder_story</x:v>
+      </x:c>
+      <x:c r="I3" s="19" t="str">
+        <x:v>Lovable's official MySafe story names the four-person team, describes the Lovable build process, and links this exact public deployment.</x:v>
+      </x:c>
+      <x:c r="J3" s="20" t="str">
+        <x:v>2025-01-17</x:v>
+      </x:c>
+      <x:c r="K3" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="L3" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
       <x:c r="M3" s="19" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="N3" s="19" t="str"/>
-      <x:c r="O3" s="19" t="str"/>
-      <x:c r="P3" s="19" t="str"/>
+        <x:v>REACHABLE</x:v>
+      </x:c>
+      <x:c r="N3" s="19" t="str">
+        <x:v>safety-sentinel-guard.lovable.app</x:v>
+      </x:c>
+      <x:c r="O3" s="19" t="str">
+        <x:v>mysafe-safety-scouts</x:v>
+      </x:c>
+      <x:c r="P3" s="19" t="str">
+        <x:v>mysafe-hackathon-team</x:v>
+      </x:c>
       <x:c r="Q3" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R3" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="S3" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="T3" s="19" t="str">
         <x:f>IF(AND(E3&lt;&gt;"",F3&lt;&gt;"",G3&lt;&gt;"",H3&lt;&gt;"",I3&lt;&gt;"",K3&lt;&gt;"",L3&lt;&gt;"",M3="REACHABLE",N3&lt;&gt;"",O3&lt;&gt;"",Q3="PASS",R3="PASS",S3="PASS"),"READY","PENDING")</x:f>
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="U3" s="19" t="str"/>
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="U3" s="19" t="str">
+        <x:v>Independent web retrieval returned the intended Safety Scouts deployment; no Development-set target, host, or tenant match found.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="17" t="str">
@@ -942,34 +966,58 @@
       <x:c r="D4" s="17" t="str">
         <x:v>Lovable</x:v>
       </x:c>
-      <x:c r="E4" s="19" t="str"/>
-      <x:c r="F4" s="19" t="str"/>
-      <x:c r="G4" s="19" t="str"/>
-      <x:c r="H4" s="19" t="str"/>
-      <x:c r="I4" s="19" t="str"/>
-      <x:c r="J4" s="20" t="str"/>
-      <x:c r="K4" s="20" t="str"/>
-      <x:c r="L4" s="20" t="str"/>
+      <x:c r="E4" s="19" t="str">
+        <x:v>AI canvas / creative workspace</x:v>
+      </x:c>
+      <x:c r="F4" s="19" t="str">
+        <x:v>https://magican.lovable.app/</x:v>
+      </x:c>
+      <x:c r="G4" s="19" t="str">
+        <x:v>https://lovable.dev/blog/zohar-vanunu-magican-ai-maker</x:v>
+      </x:c>
+      <x:c r="H4" s="19" t="str">
+        <x:v>official_builder_story</x:v>
+      </x:c>
+      <x:c r="I4" s="19" t="str">
+        <x:v>Lovable's official profile says Zohar created MagiCan through 1,500 prompts, identifies it as a Lovable project, and links this deployment.</x:v>
+      </x:c>
+      <x:c r="J4" s="20" t="str">
+        <x:v>2025-04-06</x:v>
+      </x:c>
+      <x:c r="K4" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="L4" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
       <x:c r="M4" s="19" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="N4" s="19" t="str"/>
-      <x:c r="O4" s="19" t="str"/>
-      <x:c r="P4" s="19" t="str"/>
+        <x:v>REACHABLE</x:v>
+      </x:c>
+      <x:c r="N4" s="19" t="str">
+        <x:v>magican.lovable.app</x:v>
+      </x:c>
+      <x:c r="O4" s="19" t="str">
+        <x:v>magican</x:v>
+      </x:c>
+      <x:c r="P4" s="19" t="str">
+        <x:v>zohar-vanunu-magican</x:v>
+      </x:c>
       <x:c r="Q4" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R4" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="S4" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="T4" s="19" t="str">
         <x:f>IF(AND(E4&lt;&gt;"",F4&lt;&gt;"",G4&lt;&gt;"",H4&lt;&gt;"",I4&lt;&gt;"",K4&lt;&gt;"",L4&lt;&gt;"",M4="REACHABLE",N4&lt;&gt;"",O4&lt;&gt;"",Q4="PASS",R4="PASS",S4="PASS"),"READY","PENDING")</x:f>
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="U4" s="19" t="str"/>
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="U4" s="19" t="str">
+        <x:v>Independent web retrieval returned the intended MagiCan deployment; no Development-set target, host, or tenant match found.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="17" t="str">
@@ -984,34 +1032,58 @@
       <x:c r="D5" s="17" t="str">
         <x:v>Lovable</x:v>
       </x:c>
-      <x:c r="E5" s="19" t="str"/>
-      <x:c r="F5" s="19" t="str"/>
-      <x:c r="G5" s="19" t="str"/>
-      <x:c r="H5" s="19" t="str"/>
-      <x:c r="I5" s="19" t="str"/>
-      <x:c r="J5" s="20" t="str"/>
-      <x:c r="K5" s="20" t="str"/>
-      <x:c r="L5" s="20" t="str"/>
+      <x:c r="E5" s="19" t="str">
+        <x:v>Interactive 3D experience</x:v>
+      </x:c>
+      <x:c r="F5" s="19" t="str">
+        <x:v>https://kaleidoscope-visionary.lovable.app/</x:v>
+      </x:c>
+      <x:c r="G5" s="19" t="str">
+        <x:v>https://lovable.dev/blog/2025-01-20-how-a-developer-advocate-built-stunning-3d-projects-with-lovable-dev-and-won-big</x:v>
+      </x:c>
+      <x:c r="H5" s="19" t="str">
+        <x:v>official_builder_story</x:v>
+      </x:c>
+      <x:c r="I5" s="19" t="str">
+        <x:v>Lovable's official maker interview describes Konstantin building the Kaleidoscope 3D environment with Lovable and links this exact deployment.</x:v>
+      </x:c>
+      <x:c r="J5" s="20" t="str">
+        <x:v>2025-01-20</x:v>
+      </x:c>
+      <x:c r="K5" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="L5" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
       <x:c r="M5" s="19" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="N5" s="19" t="str"/>
-      <x:c r="O5" s="19" t="str"/>
-      <x:c r="P5" s="19" t="str"/>
+        <x:v>REACHABLE</x:v>
+      </x:c>
+      <x:c r="N5" s="19" t="str">
+        <x:v>kaleidoscope-visionary.lovable.app</x:v>
+      </x:c>
+      <x:c r="O5" s="19" t="str">
+        <x:v>kaleidoscope-visionary</x:v>
+      </x:c>
+      <x:c r="P5" s="19" t="str">
+        <x:v>konstantin-zolozhkov-khvostikk</x:v>
+      </x:c>
       <x:c r="Q5" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R5" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="S5" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="T5" s="19" t="str">
         <x:f>IF(AND(E5&lt;&gt;"",F5&lt;&gt;"",G5&lt;&gt;"",H5&lt;&gt;"",I5&lt;&gt;"",K5&lt;&gt;"",L5&lt;&gt;"",M5="REACHABLE",N5&lt;&gt;"",O5&lt;&gt;"",Q5="PASS",R5="PASS",S5="PASS"),"READY","PENDING")</x:f>
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="U5" s="19" t="str"/>
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="U5" s="19" t="str">
+        <x:v>Independent web retrieval returned the intended 3D deployment; no Development-set target, host, or tenant match found.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="17" t="str">
@@ -1026,34 +1098,58 @@
       <x:c r="D6" s="17" t="str">
         <x:v>Lovable</x:v>
       </x:c>
-      <x:c r="E6" s="19" t="str"/>
-      <x:c r="F6" s="19" t="str"/>
-      <x:c r="G6" s="19" t="str"/>
-      <x:c r="H6" s="19" t="str"/>
-      <x:c r="I6" s="19" t="str"/>
-      <x:c r="J6" s="20" t="str"/>
-      <x:c r="K6" s="20" t="str"/>
-      <x:c r="L6" s="20" t="str"/>
+      <x:c r="E6" s="19" t="str">
+        <x:v>Photo-to-video creator</x:v>
+      </x:c>
+      <x:c r="F6" s="19" t="str">
+        <x:v>https://cherishable.lovable.app/</x:v>
+      </x:c>
+      <x:c r="G6" s="19" t="str">
+        <x:v>https://lovable.dev/blog/2025-01-15-lovable-christmas-hackhaton-top-10-projects</x:v>
+      </x:c>
+      <x:c r="H6" s="19" t="str">
+        <x:v>official_builder_story</x:v>
+      </x:c>
+      <x:c r="I6" s="19" t="str">
+        <x:v>Lovable's official Christmas Hackathon report identifies Cherishable as a Lovable submission, names its maker, and links this deployment.</x:v>
+      </x:c>
+      <x:c r="J6" s="20" t="str">
+        <x:v>2024-12-24</x:v>
+      </x:c>
+      <x:c r="K6" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="L6" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
       <x:c r="M6" s="19" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="N6" s="19" t="str"/>
-      <x:c r="O6" s="19" t="str"/>
-      <x:c r="P6" s="19" t="str"/>
+        <x:v>REACHABLE</x:v>
+      </x:c>
+      <x:c r="N6" s="19" t="str">
+        <x:v>cherishable.lovable.app</x:v>
+      </x:c>
+      <x:c r="O6" s="19" t="str">
+        <x:v>cherishable</x:v>
+      </x:c>
+      <x:c r="P6" s="19" t="str">
+        <x:v>tristanbob-cherishable</x:v>
+      </x:c>
       <x:c r="Q6" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R6" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="S6" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="T6" s="19" t="str">
         <x:f>IF(AND(E6&lt;&gt;"",F6&lt;&gt;"",G6&lt;&gt;"",H6&lt;&gt;"",I6&lt;&gt;"",K6&lt;&gt;"",L6&lt;&gt;"",M6="REACHABLE",N6&lt;&gt;"",O6&lt;&gt;"",Q6="PASS",R6="PASS",S6="PASS"),"READY","PENDING")</x:f>
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="U6" s="19" t="str"/>
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="U6" s="19" t="str">
+        <x:v>Independent web retrieval returned the intended Cherishable deployment; no Development-set target, host, or tenant match found.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="17" t="str">
@@ -2981,35 +3077,55 @@
       </x:c>
       <x:c r="D52" s="17" t="str"/>
       <x:c r="E52" s="19" t="str">
-        <x:v>Modern web app</x:v>
-      </x:c>
-      <x:c r="F52" s="19" t="str"/>
-      <x:c r="G52" s="19" t="str"/>
-      <x:c r="H52" s="19" t="str"/>
-      <x:c r="I52" s="19" t="str"/>
+        <x:v>Collaborative whiteboard</x:v>
+      </x:c>
+      <x:c r="F52" s="19" t="str">
+        <x:v>https://excalidraw.com/</x:v>
+      </x:c>
+      <x:c r="G52" s="19" t="str">
+        <x:v>https://github.com/excalidraw/excalidraw</x:v>
+      </x:c>
+      <x:c r="H52" s="19" t="str">
+        <x:v>repository_deployment_mapping</x:v>
+      </x:c>
+      <x:c r="I52" s="19" t="str">
+        <x:v>The official open-source repository explicitly maps its in-repository app source to excalidraw.com and exposes a multi-year, multi-contributor commit history.</x:v>
+      </x:c>
       <x:c r="J52" s="20" t="str"/>
-      <x:c r="K52" s="20" t="str"/>
-      <x:c r="L52" s="20" t="str"/>
+      <x:c r="K52" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="L52" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
       <x:c r="M52" s="19" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="N52" s="19" t="str"/>
-      <x:c r="O52" s="19" t="str"/>
-      <x:c r="P52" s="19" t="str"/>
+        <x:v>REACHABLE</x:v>
+      </x:c>
+      <x:c r="N52" s="19" t="str">
+        <x:v>excalidraw.com</x:v>
+      </x:c>
+      <x:c r="O52" s="19" t="str">
+        <x:v>excalidraw</x:v>
+      </x:c>
+      <x:c r="P52" s="19" t="str">
+        <x:v>excalidraw-community</x:v>
+      </x:c>
       <x:c r="Q52" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R52" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="S52" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="T52" s="19" t="str">
         <x:f>IF(AND(E52&lt;&gt;"",F52&lt;&gt;"",G52&lt;&gt;"",H52&lt;&gt;"",I52&lt;&gt;"",K52&lt;&gt;"",L52&lt;&gt;"",M52="REACHABLE",N52&lt;&gt;"",O52&lt;&gt;"",Q52="PASS",R52="PASS",S52="PASS"),"READY","PENDING")</x:f>
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="U52" s="19" t="str"/>
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="U52" s="19" t="str">
+        <x:v>Human control is grounded in auditable public source history and exact deployment mapping, not in the absence of AI-related product features.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="17" t="str">
@@ -3023,35 +3139,55 @@
       </x:c>
       <x:c r="D53" s="17" t="str"/>
       <x:c r="E53" s="19" t="str">
-        <x:v>Modern web app</x:v>
-      </x:c>
-      <x:c r="F53" s="19" t="str"/>
-      <x:c r="G53" s="19" t="str"/>
-      <x:c r="H53" s="19" t="str"/>
-      <x:c r="I53" s="19" t="str"/>
+        <x:v>Diagram editor</x:v>
+      </x:c>
+      <x:c r="F53" s="19" t="str">
+        <x:v>https://mermaid.live/</x:v>
+      </x:c>
+      <x:c r="G53" s="19" t="str">
+        <x:v>https://github.com/mermaid-js/mermaid-live-editor</x:v>
+      </x:c>
+      <x:c r="H53" s="19" t="str">
+        <x:v>repository_deployment_mapping</x:v>
+      </x:c>
+      <x:c r="I53" s="19" t="str">
+        <x:v>The official Mermaid Live Editor repository links mermaid.live as its live version and documents thousands of public commits and contributors.</x:v>
+      </x:c>
       <x:c r="J53" s="20" t="str"/>
-      <x:c r="K53" s="20" t="str"/>
-      <x:c r="L53" s="20" t="str"/>
+      <x:c r="K53" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="L53" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
       <x:c r="M53" s="19" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="N53" s="19" t="str"/>
-      <x:c r="O53" s="19" t="str"/>
-      <x:c r="P53" s="19" t="str"/>
+        <x:v>REACHABLE</x:v>
+      </x:c>
+      <x:c r="N53" s="19" t="str">
+        <x:v>mermaid.live</x:v>
+      </x:c>
+      <x:c r="O53" s="19" t="str">
+        <x:v>mermaid-live-editor</x:v>
+      </x:c>
+      <x:c r="P53" s="19" t="str">
+        <x:v>mermaid-js</x:v>
+      </x:c>
       <x:c r="Q53" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R53" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="S53" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="T53" s="19" t="str">
         <x:f>IF(AND(E53&lt;&gt;"",F53&lt;&gt;"",G53&lt;&gt;"",H53&lt;&gt;"",I53&lt;&gt;"",K53&lt;&gt;"",L53&lt;&gt;"",M53="REACHABLE",N53&lt;&gt;"",O53&lt;&gt;"",Q53="PASS",R53="PASS",S53="PASS"),"READY","PENDING")</x:f>
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="U53" s="19" t="str"/>
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="U53" s="19" t="str">
+        <x:v>Human control is grounded in auditable public source history and exact deployment mapping, not in the absence of AI-related product features.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="17" t="str">
@@ -3065,35 +3201,55 @@
       </x:c>
       <x:c r="D54" s="17" t="str"/>
       <x:c r="E54" s="19" t="str">
-        <x:v>Modern web app</x:v>
-      </x:c>
-      <x:c r="F54" s="19" t="str"/>
-      <x:c r="G54" s="19" t="str"/>
-      <x:c r="H54" s="19" t="str"/>
-      <x:c r="I54" s="19" t="str"/>
+        <x:v>Diagram / whiteboard app</x:v>
+      </x:c>
+      <x:c r="F54" s="19" t="str">
+        <x:v>https://app.diagrams.net/</x:v>
+      </x:c>
+      <x:c r="G54" s="19" t="str">
+        <x:v>https://github.com/jgraph/drawio</x:v>
+      </x:c>
+      <x:c r="H54" s="19" t="str">
+        <x:v>repository_deployment_mapping</x:v>
+      </x:c>
+      <x:c r="I54" s="19" t="str">
+        <x:v>The official draw.io repository identifies app.diagrams.net as the production deployment and contains the long-running client-side editor source.</x:v>
+      </x:c>
       <x:c r="J54" s="20" t="str"/>
-      <x:c r="K54" s="20" t="str"/>
-      <x:c r="L54" s="20" t="str"/>
+      <x:c r="K54" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="L54" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
       <x:c r="M54" s="19" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="N54" s="19" t="str"/>
-      <x:c r="O54" s="19" t="str"/>
-      <x:c r="P54" s="19" t="str"/>
+        <x:v>REACHABLE</x:v>
+      </x:c>
+      <x:c r="N54" s="19" t="str">
+        <x:v>diagrams.net</x:v>
+      </x:c>
+      <x:c r="O54" s="19" t="str">
+        <x:v>drawio-diagrams-net</x:v>
+      </x:c>
+      <x:c r="P54" s="19" t="str">
+        <x:v>jgraph-drawio</x:v>
+      </x:c>
       <x:c r="Q54" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R54" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="S54" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="T54" s="19" t="str">
         <x:f>IF(AND(E54&lt;&gt;"",F54&lt;&gt;"",G54&lt;&gt;"",H54&lt;&gt;"",I54&lt;&gt;"",K54&lt;&gt;"",L54&lt;&gt;"",M54="REACHABLE",N54&lt;&gt;"",O54&lt;&gt;"",Q54="PASS",R54="PASS",S54="PASS"),"READY","PENDING")</x:f>
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="U54" s="19" t="str"/>
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="U54" s="19" t="str">
+        <x:v>Human control is grounded in auditable public source history and exact deployment mapping, not in the absence of AI-related product features.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="17" t="str">
@@ -3107,35 +3263,55 @@
       </x:c>
       <x:c r="D55" s="17" t="str"/>
       <x:c r="E55" s="19" t="str">
-        <x:v>Modern web app</x:v>
-      </x:c>
-      <x:c r="F55" s="19" t="str"/>
-      <x:c r="G55" s="19" t="str"/>
-      <x:c r="H55" s="19" t="str"/>
-      <x:c r="I55" s="19" t="str"/>
+        <x:v>API development web app</x:v>
+      </x:c>
+      <x:c r="F55" s="19" t="str">
+        <x:v>https://hoppscotch.io/</x:v>
+      </x:c>
+      <x:c r="G55" s="19" t="str">
+        <x:v>https://github.com/hoppscotch/hoppscotch</x:v>
+      </x:c>
+      <x:c r="H55" s="19" t="str">
+        <x:v>repository_deployment_mapping</x:v>
+      </x:c>
+      <x:c r="I55" s="19" t="str">
+        <x:v>Hoppscotch's official open-source monorepo identifies hoppscotch.io as its web demo and documents the maintained web, desktop, and CLI project.</x:v>
+      </x:c>
       <x:c r="J55" s="20" t="str"/>
-      <x:c r="K55" s="20" t="str"/>
-      <x:c r="L55" s="20" t="str"/>
+      <x:c r="K55" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="L55" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
       <x:c r="M55" s="19" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="N55" s="19" t="str"/>
-      <x:c r="O55" s="19" t="str"/>
-      <x:c r="P55" s="19" t="str"/>
+        <x:v>REACHABLE</x:v>
+      </x:c>
+      <x:c r="N55" s="19" t="str">
+        <x:v>hoppscotch.io</x:v>
+      </x:c>
+      <x:c r="O55" s="19" t="str">
+        <x:v>hoppscotch</x:v>
+      </x:c>
+      <x:c r="P55" s="19" t="str">
+        <x:v>hoppscotch</x:v>
+      </x:c>
       <x:c r="Q55" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R55" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="S55" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="T55" s="19" t="str">
         <x:f>IF(AND(E55&lt;&gt;"",F55&lt;&gt;"",G55&lt;&gt;"",H55&lt;&gt;"",I55&lt;&gt;"",K55&lt;&gt;"",L55&lt;&gt;"",M55="REACHABLE",N55&lt;&gt;"",O55&lt;&gt;"",Q55="PASS",R55="PASS",S55="PASS"),"READY","PENDING")</x:f>
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="U55" s="19" t="str"/>
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="U55" s="19" t="str">
+        <x:v>Human control is grounded in auditable public source history and exact deployment mapping, not in the absence of AI-related product features.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="17" t="str">
@@ -3149,35 +3325,55 @@
       </x:c>
       <x:c r="D56" s="17" t="str"/>
       <x:c r="E56" s="19" t="str">
-        <x:v>Modern web app</x:v>
-      </x:c>
-      <x:c r="F56" s="19" t="str"/>
-      <x:c r="G56" s="19" t="str"/>
-      <x:c r="H56" s="19" t="str"/>
-      <x:c r="I56" s="19" t="str"/>
+        <x:v>Collaborative design tool</x:v>
+      </x:c>
+      <x:c r="F56" s="19" t="str">
+        <x:v>https://design.penpot.app/</x:v>
+      </x:c>
+      <x:c r="G56" s="19" t="str">
+        <x:v>https://github.com/penpot/penpot</x:v>
+      </x:c>
+      <x:c r="H56" s="19" t="str">
+        <x:v>repository_deployment_mapping</x:v>
+      </x:c>
+      <x:c r="I56" s="19" t="str">
+        <x:v>Penpot's official open-source repository documents the maintained collaborative design platform whose public SaaS deployment is served at design.penpot.app.</x:v>
+      </x:c>
       <x:c r="J56" s="20" t="str"/>
-      <x:c r="K56" s="20" t="str"/>
-      <x:c r="L56" s="20" t="str"/>
+      <x:c r="K56" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="L56" s="20" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
       <x:c r="M56" s="19" t="str">
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="N56" s="19" t="str"/>
-      <x:c r="O56" s="19" t="str"/>
-      <x:c r="P56" s="19" t="str"/>
+        <x:v>REACHABLE</x:v>
+      </x:c>
+      <x:c r="N56" s="19" t="str">
+        <x:v>penpot.app</x:v>
+      </x:c>
+      <x:c r="O56" s="19" t="str">
+        <x:v>penpot</x:v>
+      </x:c>
+      <x:c r="P56" s="19" t="str">
+        <x:v>kaleidos-penpot</x:v>
+      </x:c>
       <x:c r="Q56" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="R56" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="S56" s="19" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="T56" s="19" t="str">
         <x:f>IF(AND(E56&lt;&gt;"",F56&lt;&gt;"",G56&lt;&gt;"",H56&lt;&gt;"",I56&lt;&gt;"",K56&lt;&gt;"",L56&lt;&gt;"",M56="REACHABLE",N56&lt;&gt;"",O56&lt;&gt;"",Q56="PASS",R56="PASS",S56="PASS"),"READY","PENDING")</x:f>
-        <x:v>PENDING</x:v>
-      </x:c>
-      <x:c r="U56" s="19" t="str"/>
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="U56" s="19" t="str">
+        <x:v>Human control is grounded in auditable public source history and exact deployment mapping, not in the absence of AI-related product features.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="17" t="str">
@@ -5101,7 +5297,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84ac434891004a8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3de35db06dd042ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>